<commit_message>
Fill in UK events-page URLs for 128 of 186 organizations (research already done earlier this session)
</commit_message>
<xml_diff>
--- a/Sources/Event_scrapper_-_Website_completed.xlsx
+++ b/Sources/Event_scrapper_-_Website_completed.xlsx
@@ -10006,6 +10006,11 @@
           <t>Tax</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://www.tax.org.uk/events</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="28.8" customHeight="1">
       <c r="A3" t="n">
@@ -10021,6 +10026,11 @@
           <t>Tax</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://www.att.org.uk/events</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="28.8" customHeight="1">
       <c r="A4" t="n">
@@ -10036,6 +10046,11 @@
           <t>Tax / Payroll</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.cipp.org.uk/events.html</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -10051,6 +10066,11 @@
           <t>Accounting / Finance / Tax</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://www.icaew.com/learning-and-development/events</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -10066,6 +10086,11 @@
           <t>Accounting / Finance / Tax</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.accaglobal.com/learning-and-events.html</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -10081,6 +10106,11 @@
           <t>Accounting / Finance</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://www.icas.com/news-insights-events/upcoming-events</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -10096,6 +10126,11 @@
           <t>Accounting / Finance</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://www.aat.org.uk/events/search</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -10111,6 +10146,11 @@
           <t>Public Finance</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://www.cipfa.org/training/cipfa-conferences</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="28.8" customHeight="1">
       <c r="A10" t="n">
@@ -10126,6 +10166,11 @@
           <t>Finance / Treasury</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://www.treasurers.org/events</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -10141,6 +10186,11 @@
           <t>Finance / Investment</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://www.cisi.org/cisiweb2/shop/events</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -10156,6 +10206,11 @@
           <t>Investment / Finance</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://www.cfauk.org/events/events-listing</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -10171,6 +10226,11 @@
           <t>Pensions / Finance</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://www.plsa.co.uk/Events</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -10186,6 +10246,11 @@
           <t>Investment / Finance</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.theia.org/events-training</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -10201,6 +10266,11 @@
           <t>Finance / ESG</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://uksif.org/category/events/</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="28.8" customHeight="1">
       <c r="A16" t="n">
@@ -10231,6 +10301,11 @@
           <t>Governance / Legal / Finance</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://www.cgi.org.uk/events/</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -10246,6 +10321,11 @@
           <t>Finance</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://irsociety.org.uk/events</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -10261,6 +10341,11 @@
           <t>Tax / Legal</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.step.org/events</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -10276,6 +10361,11 @@
           <t>Legal</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://www.lawsociety.org.uk/events</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -10291,6 +10381,11 @@
           <t>Legal</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://www.barcouncil.org.uk/training-events/calendar.html</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -10306,6 +10401,11 @@
           <t>Legal</t>
         </is>
       </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://www.cilex.org.uk/membership/events.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -10321,6 +10421,11 @@
           <t>Legal</t>
         </is>
       </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://www.lawscot.org.uk/news-and-events/events/</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -10336,6 +10441,11 @@
           <t>Legal</t>
         </is>
       </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://lawsoc-ni.org/about-the-law-society/news-events/events</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="28.8" customHeight="1">
       <c r="A25" t="n">
@@ -10351,6 +10461,11 @@
           <t>Legal / Arbitration</t>
         </is>
       </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://www.ciarb.org/events/</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -10366,6 +10481,11 @@
           <t>International Law</t>
         </is>
       </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://www.biicl.org/events</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -10381,6 +10501,11 @@
           <t>Employment Law</t>
         </is>
       </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://www.elaweb.org.uk/future-events</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -10396,6 +10521,11 @@
           <t>Legal / Insolvency</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://www.ilauk.com/news-events/upcoming-events</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -10411,6 +10541,11 @@
           <t>Insolvency / Finance / Legal</t>
         </is>
       </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://www.r3.org.uk/events-training/</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -10426,6 +10561,11 @@
           <t>Legal</t>
         </is>
       </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://associationofcostslawyers.co.uk/events/</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -10441,6 +10581,11 @@
           <t>Legal / ADR</t>
         </is>
       </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://civilmediation.org/news-events/</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -10456,6 +10601,11 @@
           <t>Legal</t>
         </is>
       </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://www.flba.co.uk/events/</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -10471,6 +10621,11 @@
           <t>Legal / Tax</t>
         </is>
       </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://www.chba.org.uk/for-members/library/seminars</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -10486,6 +10641,11 @@
           <t>Commercial Law</t>
         </is>
       </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://www.combar.com/news-and-events/events/</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -10501,6 +10661,11 @@
           <t>Legal</t>
         </is>
       </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://tecbar.org/events/</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="28.8" customHeight="1">
       <c r="A36" t="n">
@@ -10516,6 +10681,11 @@
           <t>Credit / Finance</t>
         </is>
       </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://www.cicm.com/cicm-events/</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -10531,6 +10701,11 @@
           <t>Legal / Corporate</t>
         </is>
       </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://www.acc.com/education-events</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -10546,6 +10721,11 @@
           <t>Accounting / Finance</t>
         </is>
       </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://www.aicpa-cima.com/cpe-learning/event</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -10561,6 +10741,11 @@
           <t>Accounting / Finance</t>
         </is>
       </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://www.ifa.org.uk/cpd</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -10576,6 +10761,11 @@
           <t>Management / Finance</t>
         </is>
       </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://www.managers.org.uk/community/events/</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -10591,6 +10781,11 @@
           <t>Pensions / Finance</t>
         </is>
       </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://www.pensions-pmi.org.uk/events/</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -10606,6 +10801,11 @@
           <t>Financial Planning</t>
         </is>
       </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://events.thepfs.org/</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -10621,6 +10821,11 @@
           <t>Pensions / Legal / Finance</t>
         </is>
       </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://the-spp.co.uk/events/upcoming-events/</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -10636,6 +10841,11 @@
           <t>Tax</t>
         </is>
       </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://www.icaew.com/en/technical/tax/tax-faculty/tax-faculty-events</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -10651,6 +10861,11 @@
           <t>VAT / Tax</t>
         </is>
       </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://vpgweb.com/</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -10666,6 +10881,11 @@
           <t>Legal / Forensics</t>
         </is>
       </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://www.bafs.org.uk/events/past-events.php</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="28.8" customHeight="1">
       <c r="A47" t="n">
@@ -10681,6 +10901,11 @@
           <t>Tax</t>
         </is>
       </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://www.att.org.uk/edinburgh</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="28.8" customHeight="1">
       <c r="A48" t="n">
@@ -10696,6 +10921,11 @@
           <t>Finance / Investment</t>
         </is>
       </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://www.cisi.org/events</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="28.8" customHeight="1">
       <c r="A49" t="n">
@@ -10711,6 +10941,11 @@
           <t>Accounting / Tax</t>
         </is>
       </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://www.icaew.com/events-support</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="28.8" customHeight="1">
       <c r="A50" t="n">
@@ -10741,6 +10976,11 @@
           <t>Accounting / Finance</t>
         </is>
       </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://www.aiaworldwide.com/cpd/events/</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -10756,6 +10996,11 @@
           <t>Finance / Leasing</t>
         </is>
       </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://fla.org.uk/events/</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="28.8" customHeight="1">
       <c r="A53" t="n">
@@ -10771,6 +11016,11 @@
           <t>Legal Finance / Compliance</t>
         </is>
       </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://www.ilfm.org.uk/site/training-and-events/</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -10786,6 +11036,11 @@
           <t>Tax / Public Finance</t>
         </is>
       </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://ifs.org.uk/events</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="28.8" customHeight="1">
       <c r="A55" t="n">
@@ -10801,6 +11056,11 @@
           <t>International Tax</t>
         </is>
       </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://ifa-uk.org/events/</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -10816,6 +11076,11 @@
           <t>Finance / Financial Innovation</t>
         </is>
       </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://financeinnovationlab.org/events/</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="28.8" customHeight="1">
       <c r="A57" t="n">
@@ -10831,6 +11096,11 @@
           <t>Financial Markets</t>
         </is>
       </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://www.afme.eu/events</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -10861,6 +11131,11 @@
           <t>Financial Markets / Regulation</t>
         </is>
       </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://fmsb.com/events/</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="28.8" customHeight="1">
       <c r="A60" t="n">
@@ -10876,6 +11151,11 @@
           <t>Securities / Finance</t>
         </is>
       </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://www.islaemea.org/isla-events/</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="28.8" customHeight="1">
       <c r="A61" t="n">
@@ -10891,6 +11171,11 @@
           <t>Corporate Legal</t>
         </is>
       </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://www.acc.com/chapters-networks/chapters/europe/events-europe</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -10906,6 +11191,11 @@
           <t>Environmental Law</t>
         </is>
       </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://www.ukela.org/UKELA/UKELA/Events/Annual-Conference.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="28.8" customHeight="1">
       <c r="A63" t="n">
@@ -10921,6 +11211,11 @@
           <t>Planning / Environmental Law</t>
         </is>
       </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://peba.org.uk/news-events/</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -10936,6 +11231,11 @@
           <t>Public / Administrative Law</t>
         </is>
       </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://adminlaw.org.uk/events/</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -10966,6 +11266,11 @@
           <t>Construction Law</t>
         </is>
       </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://www.scl.org.uk/events</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -10981,6 +11286,11 @@
           <t>Technology / Legal</t>
         </is>
       </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://www.scl.org/events/event/</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="28.8" customHeight="1">
       <c r="A68" t="n">
@@ -11026,6 +11336,11 @@
           <t>IP / Commercial Law</t>
         </is>
       </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://les-bi.org/events-calendar/</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -11041,6 +11356,11 @@
           <t>Competition Law</t>
         </is>
       </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://competitionlawassociation.org.uk/events/</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="28.8" customHeight="1">
       <c r="A72" t="n">
@@ -11056,6 +11376,11 @@
           <t>Financial Services Law</t>
         </is>
       </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://fsla.org.uk/category/events/</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -11071,6 +11396,11 @@
           <t>Insolvency / Finance</t>
         </is>
       </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://insolvency-practitioners.org.uk/calendar-of-events/</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="28.8" customHeight="1">
       <c r="A74" t="n">
@@ -11086,6 +11416,11 @@
           <t>Restructuring / Finance</t>
         </is>
       </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://tma-uk.org/events/</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="28.8" customHeight="1">
       <c r="A75" t="n">
@@ -11101,6 +11436,11 @@
           <t>Credit / Financial Services</t>
         </is>
       </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://www.csa-uk.com/page/events</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -11116,6 +11456,11 @@
           <t>Risk / Finance</t>
         </is>
       </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://www.theirm.org/events/</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -11131,6 +11476,11 @@
           <t>Compliance / Financial Crime</t>
         </is>
       </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://www.int-comp.org/events/</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -11191,6 +11541,11 @@
           <t>Accounting / Tax</t>
         </is>
       </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://www.charteredaccountants.ie/professional-development/cpd-courses-and-networking-events</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="28.8" customHeight="1">
       <c r="A82" t="n">
@@ -11206,6 +11561,11 @@
           <t>Accounting / Finance</t>
         </is>
       </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://www.accaglobal.com/learning-and-events.html</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="28.8" customHeight="1">
       <c r="A83" t="n">
@@ -11221,6 +11581,11 @@
           <t>Tax</t>
         </is>
       </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>https://taxresearch.network/event/trn-26-london-registration/</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="28.8" customHeight="1">
       <c r="A84" t="n">
@@ -11266,6 +11631,11 @@
           <t>Tax / Legal / Private Client</t>
         </is>
       </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>https://www.step.org/branches/step-scotland</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="28.8" customHeight="1">
       <c r="A87" t="n">
@@ -11281,6 +11651,11 @@
           <t>Tax</t>
         </is>
       </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>https://www.att.org.uk/northern-ireland</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="28.8" customHeight="1">
       <c r="A88" t="n">
@@ -11296,6 +11671,11 @@
           <t>Business / Finance</t>
         </is>
       </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>https://www.northernirelandchamber.com/event/festival-of-business-2026/</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="28.8" customHeight="1">
       <c r="A89" t="n">
@@ -11311,6 +11691,11 @@
           <t>Financial Services</t>
         </is>
       </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>https://www.sfe.org.uk/events</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -11326,6 +11711,11 @@
           <t>Property / Finance / Legal</t>
         </is>
       </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>https://scottishpropertyfederation.org.uk/events</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -11341,6 +11731,11 @@
           <t>Arbitration / Legal</t>
         </is>
       </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>https://scottisharbitrationcentre.org/category/events-training/</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -11356,6 +11751,11 @@
           <t>Legal</t>
         </is>
       </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.co.uk/o/scottish-young-lawyers-association-1867524801</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -11386,6 +11786,11 @@
           <t>Environmental Law</t>
         </is>
       </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>https://www.ukela.org/UKELA/UKELA/Events/Annual-Conference.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="28.8" customHeight="1">
       <c r="A95" t="n">
@@ -11401,6 +11806,11 @@
           <t>Insurance Law</t>
         </is>
       </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>https://bila.org.uk/events/upcoming-events/</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -11416,6 +11826,11 @@
           <t>Pensions / Legal</t>
         </is>
       </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>http://apl-live.aptsolutions.net/calendar.php?id=5</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -11446,6 +11861,11 @@
           <t>Insolvency / Accounting</t>
         </is>
       </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://www.icaew.com/groups-and-networks/communities/restructuring-and-insolvency/restructuring-and-insolvency-community/events</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -11461,6 +11881,11 @@
           <t>Finance / Treasury</t>
         </is>
       </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>https://treasurers.ie/events</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="28.8" customHeight="1">
       <c r="A100" t="n">
@@ -11476,6 +11901,11 @@
           <t>Business / Finance</t>
         </is>
       </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>https://www.bam.ac.uk/events-landing.html</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="43.2" customHeight="1">
       <c r="A101" t="n">
@@ -11491,6 +11921,11 @@
           <t>Accounting / Finance</t>
         </is>
       </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>https://www.bafa.ac.uk/events/upcoming-events.html</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="28.8" customHeight="1">
       <c r="A102" t="n">
@@ -11506,6 +11941,11 @@
           <t>Finance / Economics</t>
         </is>
       </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>https://www.efa-finance.org/efa-annual-meeting/</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -11521,6 +11961,11 @@
           <t>Economics / Finance</t>
         </is>
       </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>https://res.org.uk/event-listing/res-2026-annual-conference/</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="28.8" customHeight="1">
       <c r="A104" t="n">
@@ -11536,6 +11981,11 @@
           <t>Economics / Finance</t>
         </is>
       </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>https://spe.org.uk/whats-on/events/</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -11551,6 +12001,11 @@
           <t>Regulation / Economics</t>
         </is>
       </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>https://ukrn.org.uk/events/</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -11566,6 +12021,11 @@
           <t>Tax / Public Finance</t>
         </is>
       </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>https://committees.parliament.uk/committee/158/treasury-committee/events/</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -11596,6 +12056,11 @@
           <t>Public Finance / Audit</t>
         </is>
       </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>https://committees.parliament.uk/committee/127/public-accounts-committee/events/</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -11611,6 +12076,11 @@
           <t>Public Policy / Finance</t>
         </is>
       </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>https://www.instituteforgovernment.org.uk/our-events</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -11626,6 +12096,11 @@
           <t>Economics / Public Finance</t>
         </is>
       </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>https://www.resolutionfoundation.org/events/</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -11656,6 +12131,11 @@
           <t>Public Finance</t>
         </is>
       </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>https://www.cipfa.org/training</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -11671,6 +12151,11 @@
           <t>Public Finance</t>
         </is>
       </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>https://publicfinancelive.org/</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -11701,6 +12186,11 @@
           <t>Tax / Public Finance</t>
         </is>
       </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>https://www.taxpayersalliance.com/events</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -11731,6 +12221,11 @@
           <t>Accounting / Finance</t>
         </is>
       </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>https://www.caba.org.uk/online-events-feedback-and-outcomes.html</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -11761,6 +12256,11 @@
           <t>Energy / Finance</t>
         </is>
       </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>https://www.biee.org/</t>
+        </is>
+      </c>
     </row>
     <row r="120" ht="28.8" customHeight="1">
       <c r="A120" t="n">
@@ -11776,6 +12276,11 @@
           <t>Energy / Regulation / Finance</t>
         </is>
       </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>https://www.energy-uk.org.uk/events/</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="28.8" customHeight="1">
       <c r="A121" t="n">
@@ -11791,6 +12296,11 @@
           <t>Industry / Finance / Regulation</t>
         </is>
       </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>https://www.makeuk.org/news-and-events/events</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -11806,6 +12316,11 @@
           <t>Business / Tax / Regulation</t>
         </is>
       </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>https://brc.org.uk/news-and-events/events/</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -11821,6 +12336,11 @@
           <t>Property / Finance / Tax</t>
         </is>
       </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>https://bpf.org.uk/events/</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -11851,6 +12371,11 @@
           <t>Property Finance</t>
         </is>
       </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>https://the-apl.com/events/</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -12331,6 +12856,11 @@
           <t>Finance / Mortgages</t>
         </is>
       </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>https://www.smp.org.uk/events/</t>
+        </is>
+      </c>
     </row>
     <row r="158" ht="28.8" customHeight="1">
       <c r="A158" t="n">
@@ -12346,6 +12876,11 @@
           <t>Property Finance / Lending</t>
         </is>
       </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>https://www.tickettailor.com/events/bdla</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -12376,6 +12911,11 @@
           <t>Business Finance / Investment</t>
         </is>
       </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>https://www.british-business-bank.co.uk/news-and-events/events</t>
+        </is>
+      </c>
     </row>
     <row r="161" ht="28.8" customHeight="1">
       <c r="A161" t="n">
@@ -12391,6 +12931,11 @@
           <t>Investment / Finance</t>
         </is>
       </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>https://ukbaa.org.uk/events/</t>
+        </is>
+      </c>
     </row>
     <row r="162" ht="28.8" customHeight="1">
       <c r="A162" t="n">
@@ -12421,6 +12966,11 @@
           <t>Pensions / Finance</t>
         </is>
       </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>https://www.pensionsuk.org.uk/Events</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -12436,6 +12986,11 @@
           <t>Actuarial / Pensions / Finance</t>
         </is>
       </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>https://aca.org.uk/events-dates/</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -12451,6 +13006,11 @@
           <t>Actuarial / Finance / Risk</t>
         </is>
       </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>https://www.actuaries.org.uk/learn-and-develop/events-calendar/events-save-date</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -12466,6 +13026,11 @@
           <t>Treasury / Finance</t>
         </is>
       </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>https://www.treasurers.org/events</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -12481,6 +13046,11 @@
           <t>International Law</t>
         </is>
       </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>https://www.biicl.org/events</t>
+        </is>
+      </c>
     </row>
     <row r="168" ht="28.8" customHeight="1">
       <c r="A168" t="n">
@@ -12496,6 +13066,11 @@
           <t>Legal</t>
         </is>
       </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>https://ilpa.org.uk/training-and-events-calendar/</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -12511,6 +13086,11 @@
           <t>Property Law</t>
         </is>
       </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>https://www.pla.org.uk/events</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -12541,6 +13121,11 @@
           <t>Accounting / Tax / Audit</t>
         </is>
       </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>https://spa.org.uk/webinars/</t>
+        </is>
+      </c>
     </row>
     <row r="172" ht="28.8" customHeight="1">
       <c r="A172" t="n">
@@ -12556,6 +13141,11 @@
           <t>Accounting / Audit</t>
         </is>
       </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>https://www.acie.org.uk/events</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -12571,6 +13161,11 @@
           <t>Tax</t>
         </is>
       </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>https://www.taxadvisers.org.uk/future-events/</t>
+        </is>
+      </c>
     </row>
     <row r="174" ht="28.8" customHeight="1">
       <c r="A174" t="n">
@@ -12586,6 +13181,11 @@
           <t>Legal Finance / Compliance / VAT</t>
         </is>
       </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>https://alca.org.uk/events/</t>
+        </is>
+      </c>
     </row>
     <row r="175" ht="28.8" customHeight="1">
       <c r="A175" t="n">
@@ -12601,6 +13201,11 @@
           <t>Legal Finance / Accounting</t>
         </is>
       </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>https://www.ilfm.org.uk/site/training-and-events/</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -12631,6 +13236,11 @@
           <t>Fraud / Finance / Compliance</t>
         </is>
       </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>https://acfeuk.co.uk/http-acfeuk-co-uk-events/</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -12646,6 +13256,11 @@
           <t>Finance / Credit / Regulation</t>
         </is>
       </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>https://fla.org.uk/events-and-training/events/</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -12676,6 +13291,11 @@
           <t>Capital Markets / Finance</t>
         </is>
       </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>https://www.afme.eu/events</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -12691,6 +13311,11 @@
           <t>Derivatives / Financial Regulation</t>
         </is>
       </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>https://www.isda.org/events</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -12721,6 +13346,11 @@
           <t>International Legal</t>
         </is>
       </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>https://www.ibanet.org/conferences</t>
+        </is>
+      </c>
     </row>
     <row r="184" ht="28.8" customHeight="1">
       <c r="A184" t="n">
@@ -12736,6 +13366,11 @@
           <t>Economics / Public Finance</t>
         </is>
       </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>https://iea.org.uk/events/</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -12749,6 +13384,11 @@
       <c r="C185" t="inlineStr">
         <is>
           <t>Tax / Public Finance</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>https://ifs.org.uk/events</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix ICAEW Tax Faculty URL, add IIA UK & Ireland events page
</commit_message>
<xml_diff>
--- a/Sources/Event_scrapper_-_Website_completed.xlsx
+++ b/Sources/Event_scrapper_-_Website_completed.xlsx
@@ -10286,6 +10286,11 @@
           <t>Audit / Finance</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://charterediia.org/events-calendar/</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="28.8" customHeight="1">
       <c r="A17" t="n">
@@ -10843,7 +10848,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.icaew.com/en/technical/tax/tax-faculty/tax-faculty-events</t>
+          <t>https://www.icaew.com/technical/tax/tax-faculty/tax-faculty-events</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Strip chatgpt.com UTM tracking param from 204 SG/UAE/AUS URLs
</commit_message>
<xml_diff>
--- a/Sources/Event_scrapper_-_Website_completed.xlsx
+++ b/Sources/Event_scrapper_-_Website_completed.xlsx
@@ -13898,7 +13898,7 @@
       </c>
       <c r="D2" s="16" t="inlineStr">
         <is>
-          <t>https://sctp.org.sg/events/Tax-Professionals?utm_source=chatgpt.com</t>
+          <t>https://sctp.org.sg/events/Tax-Professionals</t>
         </is>
       </c>
     </row>
@@ -13918,7 +13918,7 @@
       </c>
       <c r="D3" s="16" t="inlineStr">
         <is>
-          <t>https://www.isca.org.sg/member-support/events?utm_source=chatgpt.com</t>
+          <t>https://www.isca.org.sg/member-support/events</t>
         </is>
       </c>
     </row>
@@ -13938,7 +13938,7 @@
       </c>
       <c r="D4" s="16" t="inlineStr">
         <is>
-          <t>https://www.taxacademy.sg/seminars-and-conferences/?utm_source=chatgpt.com</t>
+          <t>https://www.taxacademy.sg/seminars-and-conferences/</t>
         </is>
       </c>
     </row>
@@ -13958,7 +13958,7 @@
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>https://icai.org.sg/events/recent-events?utm_source=chatgpt.com</t>
+          <t>https://icai.org.sg/events/recent-events</t>
         </is>
       </c>
     </row>
@@ -13978,7 +13978,7 @@
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>https://www.accaglobal.com/sg/en/member/cpd/events.html?utm_source=chatgpt.com</t>
+          <t>https://www.accaglobal.com/sg/en/member/cpd/events.html</t>
         </is>
       </c>
     </row>
@@ -13998,7 +13998,7 @@
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>https://www.lawsociety.org.sg/cpd-events/?utm_source=chatgpt.com</t>
+          <t>https://www.lawsociety.org.sg/cpd-events/</t>
         </is>
       </c>
     </row>
@@ -14018,7 +14018,7 @@
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>https://www.sal.org.sg/Events?utm_source=chatgpt.com</t>
+          <t>https://www.sal.org.sg/Events</t>
         </is>
       </c>
     </row>
@@ -14038,7 +14038,7 @@
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>https://www.sile.edu.sg/?utm_source=chatgpt.com</t>
+          <t>https://www.sile.edu.sg/</t>
         </is>
       </c>
     </row>
@@ -14058,7 +14058,7 @@
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>https://siac.org.sg/events?utm_source=chatgpt.com</t>
+          <t>https://siac.org.sg/events</t>
         </is>
       </c>
     </row>
@@ -14078,7 +14078,7 @@
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>https://www.sicc.gov.sg/?utm_source=chatgpt.com</t>
+          <t>https://www.sicc.gov.sg/</t>
         </is>
       </c>
     </row>
@@ -14098,7 +14098,7 @@
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>https://www.scca.org.sg/events?utm_source=chatgpt.com</t>
+          <t>https://www.scca.org.sg/events</t>
         </is>
       </c>
     </row>
@@ -14118,7 +14118,7 @@
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>https://www.sid.org.sg/events?utm_source=chatgpt.com</t>
+          <t>https://www.sid.org.sg/events</t>
         </is>
       </c>
     </row>
@@ -14138,7 +14138,7 @@
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>https://saicsa.org.sg/events/?utm_source=chatgpt.com</t>
+          <t>https://saicsa.org.sg/events/</t>
         </is>
       </c>
     </row>
@@ -14158,7 +14158,7 @@
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
-          <t>https://www.cfasocietysingapore.org/events?utm_source=chatgpt.com</t>
+          <t>https://www.cfasocietysingapore.org/events</t>
         </is>
       </c>
     </row>
@@ -14178,7 +14178,7 @@
       </c>
       <c r="D16" s="16" t="inlineStr">
         <is>
-          <t>https://imas.org.sg/events/?utm_source=chatgpt.com</t>
+          <t>https://imas.org.sg/events/</t>
         </is>
       </c>
     </row>
@@ -14198,7 +14198,7 @@
       </c>
       <c r="D17" s="16" t="inlineStr">
         <is>
-          <t>https://sias.org.sg/events/?utm_source=chatgpt.com</t>
+          <t>https://sias.org.sg/events/</t>
         </is>
       </c>
     </row>
@@ -14218,7 +14218,7 @@
       </c>
       <c r="D18" s="16" t="inlineStr">
         <is>
-          <t>https://svca.org.sg/events/?utm_source=chatgpt.com</t>
+          <t>https://svca.org.sg/events/</t>
         </is>
       </c>
     </row>
@@ -14238,7 +14238,7 @@
       </c>
       <c r="D19" s="16" t="inlineStr">
         <is>
-          <t>https://singaporefintech.org/events/?utm_source=chatgpt.com</t>
+          <t>https://singaporefintech.org/events/</t>
         </is>
       </c>
     </row>
@@ -14258,7 +14258,7 @@
       </c>
       <c r="D20" s="16" t="inlineStr">
         <is>
-          <t>https://www.abs.org.sg/events?utm_source=chatgpt.com</t>
+          <t>https://www.abs.org.sg/events</t>
         </is>
       </c>
     </row>
@@ -14278,7 +14278,7 @@
       </c>
       <c r="D21" s="16" t="inlineStr">
         <is>
-          <t>https://www.actuaries.org.sg/events/?utm_source=chatgpt.com</t>
+          <t>https://www.actuaries.org.sg/events/</t>
         </is>
       </c>
     </row>
@@ -14298,7 +14298,7 @@
       </c>
       <c r="D22" s="16" t="inlineStr">
         <is>
-          <t>https://www.sii.org.sg/events?utm_source=chatgpt.com</t>
+          <t>https://www.sii.org.sg/events</t>
         </is>
       </c>
     </row>
@@ -14318,7 +14318,7 @@
       </c>
       <c r="D23" s="16" t="inlineStr">
         <is>
-          <t>https://www.fpas.org.sg/events/?utm_source=chatgpt.com</t>
+          <t>https://www.fpas.org.sg/events/</t>
         </is>
       </c>
     </row>
@@ -14338,7 +14338,7 @@
       </c>
       <c r="D24" s="16" t="inlineStr">
         <is>
-          <t>https://www.acra.gov.sg/news-events/event-highlights/?utm_source=chatgpt.com</t>
+          <t>https://www.acra.gov.sg/news-events/event-highlights/</t>
         </is>
       </c>
     </row>
@@ -14358,7 +14358,7 @@
       </c>
       <c r="D25" s="16" t="inlineStr">
         <is>
-          <t>https://www.iras.gov.sg/?utm_source=chatgpt.com</t>
+          <t>https://www.iras.gov.sg/</t>
         </is>
       </c>
     </row>
@@ -14378,7 +14378,7 @@
       </c>
       <c r="D26" s="16" t="inlineStr">
         <is>
-          <t>https://www.mas.gov.sg/news/events?utm_source=chatgpt.com</t>
+          <t>https://www.mas.gov.sg/news/events</t>
         </is>
       </c>
     </row>
@@ -14398,7 +14398,7 @@
       </c>
       <c r="D27" s="16" t="inlineStr">
         <is>
-          <t>https://www.ipos.gov.sg/events?utm_source=chatgpt.com</t>
+          <t>https://www.ipos.gov.sg/events</t>
         </is>
       </c>
     </row>
@@ -14418,7 +14418,7 @@
       </c>
       <c r="D28" s="16" t="inlineStr">
         <is>
-          <t>https://www.mof.gov.sg/news-publications/events?utm_source=chatgpt.com</t>
+          <t>https://www.mof.gov.sg/news-publications/events</t>
         </is>
       </c>
     </row>
@@ -14438,7 +14438,7 @@
       </c>
       <c r="D29" s="16" t="inlineStr">
         <is>
-          <t>https://www.sbf.org.sg/events?utm_source=chatgpt.com</t>
+          <t>https://www.sbf.org.sg/events</t>
         </is>
       </c>
     </row>
@@ -14458,7 +14458,7 @@
       </c>
       <c r="D30" s="16" t="inlineStr">
         <is>
-          <t>https://sicc.com.sg/events/?utm_source=chatgpt.com</t>
+          <t>https://sicc.com.sg/events/</t>
         </is>
       </c>
     </row>
@@ -14478,7 +14478,7 @@
       </c>
       <c r="D31" s="16" t="inlineStr">
         <is>
-          <t>https://www.sccci.org.sg/events/?utm_source=chatgpt.com</t>
+          <t>https://www.sccci.org.sg/events/</t>
         </is>
       </c>
     </row>
@@ -14498,7 +14498,7 @@
       </c>
       <c r="D32" s="16" t="inlineStr">
         <is>
-          <t>https://asme.org.sg/events/?utm_source=chatgpt.com</t>
+          <t>https://asme.org.sg/events/</t>
         </is>
       </c>
     </row>
@@ -14518,7 +14518,7 @@
       </c>
       <c r="D33" s="16" t="inlineStr">
         <is>
-          <t>https://www.smfederation.org.sg/events/?utm_source=chatgpt.com</t>
+          <t>https://www.smfederation.org.sg/events/</t>
         </is>
       </c>
     </row>
@@ -14538,7 +14538,7 @@
       </c>
       <c r="D34" s="16" t="inlineStr">
         <is>
-          <t>https://www.sla.org.sg/events/?utm_source=chatgpt.com</t>
+          <t>https://www.sla.org.sg/events/</t>
         </is>
       </c>
     </row>
@@ -14558,7 +14558,7 @@
       </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
-          <t>https://www.enterprisesg.gov.sg/events?utm_source=chatgpt.com</t>
+          <t>https://www.enterprisesg.gov.sg/events</t>
         </is>
       </c>
     </row>
@@ -14578,7 +14578,7 @@
       </c>
       <c r="D36" s="16" t="inlineStr">
         <is>
-          <t>https://www.edb.gov.sg/en/events.html?utm_source=chatgpt.com</t>
+          <t>https://www.edb.gov.sg/en/events.html</t>
         </is>
       </c>
     </row>
@@ -14598,7 +14598,7 @@
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>https://www.step.org/singapore/events?utm_source=chatgpt.com</t>
+          <t>https://www.step.org/singapore/events</t>
         </is>
       </c>
     </row>
@@ -14618,7 +14618,7 @@
       </c>
       <c r="D38" s="16" t="inlineStr">
         <is>
-          <t>https://www.ifa.nl/events?utm_source=chatgpt.com</t>
+          <t>https://www.ifa.nl/events</t>
         </is>
       </c>
     </row>
@@ -14638,7 +14638,7 @@
       </c>
       <c r="D39" s="16" t="inlineStr">
         <is>
-          <t>https://www.taxacademy.sg/stari/?utm_source=chatgpt.com</t>
+          <t>https://www.taxacademy.sg/stari/</t>
         </is>
       </c>
     </row>
@@ -14658,7 +14658,7 @@
       </c>
       <c r="D40" s="16" t="inlineStr">
         <is>
-          <t>https://www.ivass.org.sg/events?utm_source=chatgpt.com</t>
+          <t>https://www.ivass.org.sg/events</t>
         </is>
       </c>
     </row>
@@ -14678,7 +14678,7 @@
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>https://scma.org.sg/events/?utm_source=chatgpt.com</t>
+          <t>https://scma.org.sg/events/</t>
         </is>
       </c>
     </row>
@@ -14698,7 +14698,7 @@
       </c>
       <c r="D42" s="16" t="inlineStr">
         <is>
-          <t>https://www.smc.org.sg/events?utm_source=chatgpt.com</t>
+          <t>https://www.smc.org.sg/events</t>
         </is>
       </c>
     </row>
@@ -14718,7 +14718,7 @@
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>https://sicc.gov.sg/?utm_source=chatgpt.com</t>
+          <t>https://sicc.gov.sg/</t>
         </is>
       </c>
     </row>
@@ -14738,7 +14738,7 @@
       </c>
       <c r="D44" s="16" t="inlineStr">
         <is>
-          <t>https://www.scs.org.sg/events?utm_source=chatgpt.com</t>
+          <t>https://www.scs.org.sg/events</t>
         </is>
       </c>
     </row>
@@ -14758,7 +14758,7 @@
       </c>
       <c r="D45" s="16" t="inlineStr">
         <is>
-          <t>https://www.sim.edu.sg/?utm_source=chatgpt.com</t>
+          <t>https://www.sim.edu.sg/</t>
         </is>
       </c>
     </row>
@@ -14778,7 +14778,7 @@
       </c>
       <c r="D46" s="16" t="inlineStr">
         <is>
-          <t>https://www.shri.org.sg/events?utm_source=chatgpt.com</t>
+          <t>https://www.shri.org.sg/events</t>
         </is>
       </c>
     </row>
@@ -14798,7 +14798,7 @@
       </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>https://mis.org.sg/events/?utm_source=chatgpt.com</t>
+          <t>https://mis.org.sg/events/</t>
         </is>
       </c>
     </row>
@@ -14818,7 +14818,7 @@
       </c>
       <c r="D48" s="16" t="inlineStr">
         <is>
-          <t>https://www.sipmm.edu.sg/events/?utm_source=chatgpt.com</t>
+          <t>https://www.sipmm.edu.sg/events/</t>
         </is>
       </c>
     </row>
@@ -14838,7 +14838,7 @@
       </c>
       <c r="D49" s="16" t="inlineStr">
         <is>
-          <t>https://ccls.smu.edu.sg/events?utm_source=chatgpt.com</t>
+          <t>https://ccls.smu.edu.sg/events</t>
         </is>
       </c>
     </row>
@@ -14858,7 +14858,7 @@
       </c>
       <c r="D50" s="16" t="inlineStr">
         <is>
-          <t>https://law.smu.edu.sg/events?utm_source=chatgpt.com</t>
+          <t>https://law.smu.edu.sg/events</t>
         </is>
       </c>
     </row>
@@ -14878,7 +14878,7 @@
       </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
-          <t>https://caidg.smu.edu.sg/events?utm_source=chatgpt.com</t>
+          <t>https://caidg.smu.edu.sg/events</t>
         </is>
       </c>
     </row>
@@ -14898,7 +14898,7 @@
       </c>
       <c r="D52" s="16" t="inlineStr">
         <is>
-          <t>https://act.org.sg/events/?utm_source=chatgpt.com</t>
+          <t>https://act.org.sg/events/</t>
         </is>
       </c>
     </row>
@@ -14918,7 +14918,7 @@
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>https://www.rimas.org.sg/?utm_source=chatgpt.com</t>
+          <t>https://www.rimas.org.sg/</t>
         </is>
       </c>
     </row>
@@ -14938,7 +14938,7 @@
       </c>
       <c r="D54" s="16" t="inlineStr">
         <is>
-          <t>https://iia.org.sg/Home?utm_source=chatgpt.com</t>
+          <t>https://iia.org.sg/Home</t>
         </is>
       </c>
     </row>
@@ -14958,7 +14958,7 @@
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>https://engage.isaca.org/singaporechapter/events?utm_source=chatgpt.com</t>
+          <t>https://engage.isaca.org/singaporechapter/events</t>
         </is>
       </c>
     </row>
@@ -14978,7 +14978,7 @@
       </c>
       <c r="D56" s="16" t="inlineStr">
         <is>
-          <t>https://www.isc2chapter.sg/events?utm_source=chatgpt.com</t>
+          <t>https://www.isc2chapter.sg/events</t>
         </is>
       </c>
     </row>
@@ -14998,7 +14998,7 @@
       </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
-          <t>https://siarb.org.sg/?utm_source=chatgpt.com</t>
+          <t>https://siarb.org.sg/</t>
         </is>
       </c>
     </row>
@@ -15018,7 +15018,7 @@
       </c>
       <c r="D58" s="16" t="inlineStr">
         <is>
-          <t>https://ciarbsingapore.wildapricot.org/events?utm_source=chatgpt.com</t>
+          <t>https://ciarbsingapore.wildapricot.org/events</t>
         </is>
       </c>
     </row>
@@ -15038,7 +15038,7 @@
       </c>
       <c r="D59" s="16" t="inlineStr">
         <is>
-          <t>https://www.acc.com/webview/events?utm_source=chatgpt.com</t>
+          <t>https://www.acc.com/webview/events</t>
         </is>
       </c>
     </row>
@@ -15058,7 +15058,7 @@
       </c>
       <c r="D60" s="16" t="inlineStr">
         <is>
-          <t>https://www.fwasg.org/events/Default.aspx?utm_source=chatgpt.com</t>
+          <t>https://www.fwasg.org/events/Default.aspx</t>
         </is>
       </c>
     </row>
@@ -15078,7 +15078,7 @@
       </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
-          <t>https://caia.org/chapter-locations/caia-chapter-singapore/?utm_source=chatgpt.com</t>
+          <t>https://caia.org/chapter-locations/caia-chapter-singapore/</t>
         </is>
       </c>
     </row>
@@ -15098,7 +15098,7 @@
       </c>
       <c r="D62" s="16" t="inlineStr">
         <is>
-          <t>https://www.isda.org/location/singapore/?utm_source=chatgpt.com</t>
+          <t>https://www.isda.org/location/singapore/</t>
         </is>
       </c>
     </row>
@@ -15118,7 +15118,7 @@
       </c>
       <c r="D63" s="16" t="inlineStr">
         <is>
-          <t>https://www.traceinternational.org/events?utm_source=chatgpt.com</t>
+          <t>https://www.traceinternational.org/events</t>
         </is>
       </c>
     </row>
@@ -15138,7 +15138,7 @@
       </c>
       <c r="D64" s="16" t="inlineStr">
         <is>
-          <t>https://members.agrc.org/events/event_list.asp?group=258545&amp;show=&amp;utm_source=chatgpt.com</t>
+          <t>https://members.agrc.org/events/event_list.asp?group=258545</t>
         </is>
       </c>
     </row>
@@ -15158,7 +15158,7 @@
       </c>
       <c r="D65" s="16" t="inlineStr">
         <is>
-          <t>https://iapp.org/events/?utm_source=chatgpt.com</t>
+          <t>https://iapp.org/events/</t>
         </is>
       </c>
     </row>
@@ -15178,7 +15178,7 @@
       </c>
       <c r="D66" s="16" t="inlineStr">
         <is>
-          <t>https://www.int-comp.org/events/?utm_source=chatgpt.com</t>
+          <t>https://www.int-comp.org/events/</t>
         </is>
       </c>
     </row>
@@ -15198,7 +15198,7 @@
       </c>
       <c r="D67" s="16" t="inlineStr">
         <is>
-          <t>https://www.acfe.com/?utm_source=chatgpt.com</t>
+          <t>https://www.acfe.com/</t>
         </is>
       </c>
     </row>
@@ -15218,7 +15218,7 @@
       </c>
       <c r="D68" s="16" t="inlineStr">
         <is>
-          <t>https://www.acams.org/en/events?utm_source=chatgpt.com</t>
+          <t>https://www.acams.org/en/events</t>
         </is>
       </c>
     </row>
@@ -15238,7 +15238,7 @@
       </c>
       <c r="D69" s="16" t="inlineStr">
         <is>
-          <t>https://www.acga-asia.org/events.php?utm_source=chatgpt.com</t>
+          <t>https://www.acga-asia.org/events.php</t>
         </is>
       </c>
     </row>
@@ -15258,7 +15258,7 @@
       </c>
       <c r="D70" s="16" t="inlineStr">
         <is>
-          <t>https://www.reitas.sg/events/upcoming-events/?utm_source=chatgpt.com</t>
+          <t>https://www.reitas.sg/events/upcoming-events/</t>
         </is>
       </c>
     </row>
@@ -15278,7 +15278,7 @@
       </c>
       <c r="D71" s="16" t="inlineStr">
         <is>
-          <t>https://singaporefintech.org/event/?utm_source=chatgpt.com</t>
+          <t>https://singaporefintech.org/event/</t>
         </is>
       </c>
     </row>
@@ -15298,7 +15298,7 @@
       </c>
       <c r="D72" s="16" t="inlineStr">
         <is>
-          <t>https://www.ibf.org.sg/?utm_source=chatgpt.com</t>
+          <t>https://www.ibf.org.sg/</t>
         </is>
       </c>
     </row>
@@ -15318,7 +15318,7 @@
       </c>
       <c r="D73" s="16" t="inlineStr">
         <is>
-          <t>https://www.aima.org/events/aima-conferences-information/aima-singapore-forum.html?utm_source=chatgpt.com</t>
+          <t>https://www.aima.org/events/aima-conferences-information/aima-singapore-forum.html</t>
         </is>
       </c>
     </row>
@@ -15338,7 +15338,7 @@
       </c>
       <c r="D74" s="16" t="inlineStr">
         <is>
-          <t>https://www.theirm.org/events/?utm_source=chatgpt.com</t>
+          <t>https://www.theirm.org/events/</t>
         </is>
       </c>
     </row>
@@ -15358,7 +15358,7 @@
       </c>
       <c r="D75" s="16" t="inlineStr">
         <is>
-          <t>https://www.treasurers.org/events-and-networking/upcoming-events/?utm_source=chatgpt.com</t>
+          <t>https://www.treasurers.org/events-and-networking/upcoming-events/</t>
         </is>
       </c>
     </row>
@@ -15378,7 +15378,7 @@
       </c>
       <c r="D76" s="16" t="inlineStr">
         <is>
-          <t>https://events2go.iccwbo.org/?utm_source=chatgpt.com</t>
+          <t>https://events2go.iccwbo.org/</t>
         </is>
       </c>
     </row>
@@ -15398,7 +15398,7 @@
       </c>
       <c r="D77" s="16" t="inlineStr">
         <is>
-          <t>https://www.ibanet.org/conferences-events?utm_source=chatgpt.com</t>
+          <t>https://www.ibanet.org/conferences-events</t>
         </is>
       </c>
     </row>
@@ -15418,7 +15418,7 @@
       </c>
       <c r="D78" s="16" t="inlineStr">
         <is>
-          <t>https://www.ifa.nl/events?utm_source=chatgpt.com</t>
+          <t>https://www.ifa.nl/events</t>
         </is>
       </c>
     </row>
@@ -15438,7 +15438,7 @@
       </c>
       <c r="D79" s="16" t="inlineStr">
         <is>
-          <t>https://www.step.org/events?utm_source=chatgpt.com</t>
+          <t>https://www.step.org/events</t>
         </is>
       </c>
     </row>
@@ -15458,7 +15458,7 @@
       </c>
       <c r="D80" s="16" t="inlineStr">
         <is>
-          <t>https://www.internationaltaxreview.com/events?utm_source=chatgpt.com</t>
+          <t>https://www.internationaltaxreview.com/events</t>
         </is>
       </c>
     </row>
@@ -15478,7 +15478,7 @@
       </c>
       <c r="D81" s="16" t="inlineStr">
         <is>
-          <t>https://www.ibanet.org/conferences-events?utm_source=chatgpt.com</t>
+          <t>https://www.ibanet.org/conferences-events</t>
         </is>
       </c>
     </row>
@@ -15498,7 +15498,7 @@
       </c>
       <c r="D82" s="16" t="inlineStr">
         <is>
-          <t>https://www.aija.org/events/?utm_source=chatgpt.com</t>
+          <t>https://www.aija.org/events/</t>
         </is>
       </c>
     </row>
@@ -15518,7 +15518,7 @@
       </c>
       <c r="D83" s="16" t="inlineStr">
         <is>
-          <t>https://www.ipba.org/events/?utm_source=chatgpt.com</t>
+          <t>https://www.ipba.org/events/</t>
         </is>
       </c>
     </row>
@@ -15538,7 +15538,7 @@
       </c>
       <c r="D84" s="16" t="inlineStr">
         <is>
-          <t>https://www.uianet.org/en/events?utm_source=chatgpt.com</t>
+          <t>https://www.uianet.org/en/events</t>
         </is>
       </c>
     </row>
@@ -15558,7 +15558,7 @@
       </c>
       <c r="D85" s="16" t="inlineStr">
         <is>
-          <t>https://www.worldcc.com/Events?utm_source=chatgpt.com</t>
+          <t>https://www.worldcc.com/Events</t>
         </is>
       </c>
     </row>
@@ -15578,7 +15578,7 @@
       </c>
       <c r="D86" s="16" t="inlineStr">
         <is>
-          <t>https://www.cips.org/events?utm_source=chatgpt.com</t>
+          <t>https://www.cips.org/events</t>
         </is>
       </c>
     </row>
@@ -15598,7 +15598,7 @@
       </c>
       <c r="D87" s="16" t="inlineStr">
         <is>
-          <t>https://www.ismworld.org/events/?utm_source=chatgpt.com</t>
+          <t>https://www.ismworld.org/events/</t>
         </is>
       </c>
     </row>
@@ -15618,7 +15618,7 @@
       </c>
       <c r="D88" s="16" t="inlineStr">
         <is>
-          <t>https://www.afponline.org/events?utm_source=chatgpt.com</t>
+          <t>https://www.afponline.org/events</t>
         </is>
       </c>
     </row>
@@ -15638,7 +15638,7 @@
       </c>
       <c r="D89" s="16" t="inlineStr">
         <is>
-          <t>https://www.garp.org/events?utm_source=chatgpt.com</t>
+          <t>https://www.garp.org/events</t>
         </is>
       </c>
     </row>
@@ -15658,7 +15658,7 @@
       </c>
       <c r="D90" s="16" t="inlineStr">
         <is>
-          <t>https://www.prmia.org/events?utm_source=chatgpt.com</t>
+          <t>https://www.prmia.org/events</t>
         </is>
       </c>
     </row>
@@ -15678,7 +15678,7 @@
       </c>
       <c r="D91" s="16" t="inlineStr">
         <is>
-          <t>https://www.gacp.org/events?utm_source=chatgpt.com</t>
+          <t>https://www.gacp.org/events</t>
         </is>
       </c>
     </row>
@@ -15698,7 +15698,7 @@
       </c>
       <c r="D92" s="16" t="inlineStr">
         <is>
-          <t>https://www.acfcs.org/events?utm_source=chatgpt.com</t>
+          <t>https://www.acfcs.org/events</t>
         </is>
       </c>
     </row>
@@ -15718,7 +15718,7 @@
       </c>
       <c r="D93" s="16" t="inlineStr">
         <is>
-          <t>https://www.iais.org/activities-meetings/?utm_source=chatgpt.com</t>
+          <t>https://www.iais.org/activities-meetings/</t>
         </is>
       </c>
     </row>
@@ -15738,7 +15738,7 @@
       </c>
       <c r="D94" s="16" t="inlineStr">
         <is>
-          <t>https://www.iosco.org/events/?utm_source=chatgpt.com</t>
+          <t>https://www.iosco.org/events/</t>
         </is>
       </c>
     </row>
@@ -15758,7 +15758,7 @@
       </c>
       <c r="D95" s="16" t="inlineStr">
         <is>
-          <t>https://www.internationalinsuranceprofessionals.org/events?utm_source=chatgpt.com</t>
+          <t>https://www.internationalinsuranceprofessionals.org/events</t>
         </is>
       </c>
     </row>
@@ -15778,7 +15778,7 @@
       </c>
       <c r="D96" s="16" t="inlineStr">
         <is>
-          <t>https://www.globalreporting.org/events/?utm_source=chatgpt.com</t>
+          <t>https://www.globalreporting.org/events/</t>
         </is>
       </c>
     </row>
@@ -15798,7 +15798,7 @@
       </c>
       <c r="D97" s="16" t="inlineStr">
         <is>
-          <t>https://www.ifrs.org/news-and-events/events/?utm_source=chatgpt.com</t>
+          <t>https://www.ifrs.org/news-and-events/events/</t>
         </is>
       </c>
     </row>
@@ -15818,7 +15818,7 @@
       </c>
       <c r="D98" s="16" t="inlineStr">
         <is>
-          <t>https://www.ifrs.org/news-and-events/events/?utm_source=chatgpt.com</t>
+          <t>https://www.ifrs.org/news-and-events/events/</t>
         </is>
       </c>
     </row>
@@ -15838,7 +15838,7 @@
       </c>
       <c r="D99" s="16" t="inlineStr">
         <is>
-          <t>https://www.weforum.org/events/?utm_source=chatgpt.com</t>
+          <t>https://www.weforum.org/events/</t>
         </is>
       </c>
     </row>
@@ -15858,7 +15858,7 @@
       </c>
       <c r="D100" s="16" t="inlineStr">
         <is>
-          <t>https://uncitral.un.org/en/events?utm_source=chatgpt.com</t>
+          <t>https://uncitral.un.org/en/events</t>
         </is>
       </c>
     </row>
@@ -19116,7 +19116,7 @@
       </c>
       <c r="D52" s="16" t="inlineStr">
         <is>
-          <t>https://www.aopauae.com/events?utm_source=chatgpt.com</t>
+          <t>https://www.aopauae.com/events</t>
         </is>
       </c>
     </row>
@@ -19136,7 +19136,7 @@
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>https://mail.aaa4uae.ae/site/en/eaaa?utm_source=chatgpt.com</t>
+          <t>https://mail.aaa4uae.ae/site/en/eaaa</t>
         </is>
       </c>
     </row>
@@ -19156,7 +19156,7 @@
       </c>
       <c r="D54" s="16" t="inlineStr">
         <is>
-          <t>https://www.garp.org/membership/chapter/united-arab-emirates?utm_source=chatgpt.com</t>
+          <t>https://www.garp.org/membership/chapter/united-arab-emirates</t>
         </is>
       </c>
     </row>
@@ -19176,7 +19176,7 @@
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>https://www.acfe.com/calendar?utm_source=chatgpt.com</t>
+          <t>https://www.acfe.com/calendar</t>
         </is>
       </c>
     </row>
@@ -19196,7 +19196,7 @@
       </c>
       <c r="D56" s="16" t="inlineStr">
         <is>
-          <t>https://slba.ae/events/?utm_source=chatgpt.com</t>
+          <t>https://slba.ae/events/</t>
         </is>
       </c>
     </row>
@@ -19216,7 +19216,7 @@
       </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
-          <t>https://academy.adgm.com/events/?utm_source=chatgpt.com</t>
+          <t>https://academy.adgm.com/events/</t>
         </is>
       </c>
     </row>
@@ -19236,7 +19236,7 @@
       </c>
       <c r="D58" s="16" t="inlineStr">
         <is>
-          <t>https://ajmanchamber.ae/en/archives/exhibitions-conferences/?utm_source=chatgpt.com</t>
+          <t>https://ajmanchamber.ae/en/archives/exhibitions-conferences/</t>
         </is>
       </c>
     </row>
@@ -19256,7 +19256,7 @@
       </c>
       <c r="D59" s="16" t="inlineStr">
         <is>
-          <t>https://rakchamber.ae/?utm_source=chatgpt.com</t>
+          <t>https://rakchamber.ae/</t>
         </is>
       </c>
     </row>
@@ -19276,7 +19276,7 @@
       </c>
       <c r="D60" s="16" t="inlineStr">
         <is>
-          <t>https://www.fujairahchamber.ae/?utm_source=chatgpt.com</t>
+          <t>https://www.fujairahchamber.ae/</t>
         </is>
       </c>
     </row>
@@ -19296,7 +19296,7 @@
       </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
-          <t>https://uaqchamber.ae/?utm_source=chatgpt.com</t>
+          <t>https://uaqchamber.ae/</t>
         </is>
       </c>
     </row>
@@ -19316,7 +19316,7 @@
       </c>
       <c r="D62" s="16" t="inlineStr">
         <is>
-          <t>https://www.irishbusinessnetwork.org/events/?utm_source=chatgpt.com</t>
+          <t>https://www.irishbusinessnetwork.org/events/</t>
         </is>
       </c>
     </row>
@@ -19336,7 +19336,7 @@
       </c>
       <c r="D63" s="16" t="inlineStr">
         <is>
-          <t>https://www.sbcuae.se/events?utm_source=chatgpt.com</t>
+          <t>https://www.sbcuae.se/events</t>
         </is>
       </c>
     </row>
@@ -19356,7 +19356,7 @@
       </c>
       <c r="D64" s="16" t="inlineStr">
         <is>
-          <t>https://www.bbc-uae.com/events?utm_source=chatgpt.com</t>
+          <t>https://www.bbc-uae.com/events</t>
         </is>
       </c>
     </row>
@@ -19376,7 +19376,7 @@
       </c>
       <c r="D65" s="16" t="inlineStr">
         <is>
-          <t>https://www.sbcuae.org/events?utm_source=chatgpt.com</t>
+          <t>https://www.sbcuae.org/events</t>
         </is>
       </c>
     </row>
@@ -19396,7 +19396,7 @@
       </c>
       <c r="D66" s="16" t="inlineStr">
         <is>
-          <t>https://www.diac.com/en/events/?utm_source=chatgpt.com</t>
+          <t>https://www.diac.com/en/events/</t>
         </is>
       </c>
     </row>
@@ -19416,7 +19416,7 @@
       </c>
       <c r="D67" s="16" t="inlineStr">
         <is>
-          <t>https://www.adjd.gov.ae/EN/Pages/Events.aspx?utm_source=chatgpt.com</t>
+          <t>https://www.adjd.gov.ae/EN/Pages/Events.aspx</t>
         </is>
       </c>
     </row>
@@ -19436,7 +19436,7 @@
       </c>
       <c r="D68" s="16" t="inlineStr">
         <is>
-          <t>https://www.dld.gov.ae/?utm_source=chatgpt.com</t>
+          <t>https://www.dld.gov.ae/</t>
         </is>
       </c>
     </row>
@@ -19456,7 +19456,7 @@
       </c>
       <c r="D69" s="16" t="inlineStr">
         <is>
-          <t>https://www.emirateslegalnetwork.com/events?utm_source=chatgpt.com</t>
+          <t>https://www.emirateslegalnetwork.com/events</t>
         </is>
       </c>
     </row>
@@ -19476,7 +19476,7 @@
       </c>
       <c r="D70" s="16" t="inlineStr">
         <is>
-          <t>https://cms.law/en/are/events?utm_source=chatgpt.com</t>
+          <t>https://cms.law/en/are/events</t>
         </is>
       </c>
     </row>
@@ -19496,7 +19496,7 @@
       </c>
       <c r="D71" s="16" t="inlineStr">
         <is>
-          <t>https://mena.thomsonreuters.com/en/events.html?utm_source=chatgpt.com</t>
+          <t>https://mena.thomsonreuters.com/en/events.html</t>
         </is>
       </c>
     </row>
@@ -19516,7 +19516,7 @@
       </c>
       <c r="D72" s="16" t="inlineStr">
         <is>
-          <t>https://www.bakertilly.ae/events?utm_source=chatgpt.com</t>
+          <t>https://www.bakertilly.ae/events</t>
         </is>
       </c>
     </row>
@@ -19536,7 +19536,7 @@
       </c>
       <c r="D73" s="16" t="inlineStr">
         <is>
-          <t>https://www.grantthornton.ae/events/?utm_source=chatgpt.com</t>
+          <t>https://www.grantthornton.ae/events/</t>
         </is>
       </c>
     </row>
@@ -19556,7 +19556,7 @@
       </c>
       <c r="D74" s="16" t="inlineStr">
         <is>
-          <t>https://www.crowe.com/ae/events?utm_source=chatgpt.com</t>
+          <t>https://www.crowe.com/ae/events</t>
         </is>
       </c>
     </row>
@@ -19576,7 +19576,7 @@
       </c>
       <c r="D75" s="16" t="inlineStr">
         <is>
-          <t>https://www.deloitte.com/middle-east/en/events.html?utm_source=chatgpt.com</t>
+          <t>https://www.deloitte.com/middle-east/en/events.html</t>
         </is>
       </c>
     </row>
@@ -19596,7 +19596,7 @@
       </c>
       <c r="D76" s="16" t="inlineStr">
         <is>
-          <t>https://www.bdo.ae/en-gb/events?utm_source=chatgpt.com</t>
+          <t>https://www.bdo.ae/en-gb/events</t>
         </is>
       </c>
     </row>
@@ -19616,7 +19616,7 @@
       </c>
       <c r="D77" s="16" t="inlineStr">
         <is>
-          <t>https://kpmg.com/ae/en/home/events.html?utm_source=chatgpt.com</t>
+          <t>https://kpmg.com/ae/en/home/events.html</t>
         </is>
       </c>
     </row>
@@ -19636,7 +19636,7 @@
       </c>
       <c r="D78" s="16" t="inlineStr">
         <is>
-          <t>https://www.pwc.com/m1/en/events.html?utm_source=chatgpt.com</t>
+          <t>https://www.pwc.com/m1/en/events.html</t>
         </is>
       </c>
     </row>
@@ -19656,7 +19656,7 @@
       </c>
       <c r="D79" s="16" t="inlineStr">
         <is>
-          <t>https://www.ey.com/en_ae/events?utm_source=chatgpt.com</t>
+          <t>https://www.ey.com/en_ae/events</t>
         </is>
       </c>
     </row>
@@ -19676,7 +19676,7 @@
       </c>
       <c r="D80" s="16" t="inlineStr">
         <is>
-          <t>https://uaeiaa.org/events-calendar?utm_source=chatgpt.com</t>
+          <t>https://uaeiaa.org/events-calendar</t>
         </is>
       </c>
     </row>
@@ -19696,7 +19696,7 @@
       </c>
       <c r="D81" s="16" t="inlineStr">
         <is>
-          <t>https://www.cisi.org/cisiweb2/events?utm_source=chatgpt.com</t>
+          <t>https://www.cisi.org/cisiweb2/events</t>
         </is>
       </c>
     </row>
@@ -19716,7 +19716,7 @@
       </c>
       <c r="D82" s="16" t="inlineStr">
         <is>
-          <t>https://www.globalethicalfinance.org/our-events/?utm_source=chatgpt.com</t>
+          <t>https://www.globalethicalfinance.org/our-events/</t>
         </is>
       </c>
     </row>
@@ -19736,7 +19736,7 @@
       </c>
       <c r="D83" s="16" t="inlineStr">
         <is>
-          <t>https://www.dsig.ae/upcoming-events/?utm_source=chatgpt.com</t>
+          <t>https://www.dsig.ae/upcoming-events/</t>
         </is>
       </c>
     </row>
@@ -19756,7 +19756,7 @@
       </c>
       <c r="D84" s="16" t="inlineStr">
         <is>
-          <t>https://academy.adgm.com/events/?utm_source=chatgpt.com</t>
+          <t>https://academy.adgm.com/events/</t>
         </is>
       </c>
     </row>
@@ -19776,7 +19776,7 @@
       </c>
       <c r="D85" s="16" t="inlineStr">
         <is>
-          <t>https://moiat.gov.ae/en/media-center/events?utm_source=chatgpt.com</t>
+          <t>https://moiat.gov.ae/en/media-center/events</t>
         </is>
       </c>
     </row>
@@ -19796,7 +19796,7 @@
       </c>
       <c r="D86" s="16" t="inlineStr">
         <is>
-          <t>https://rakchamber.ae/?utm_source=chatgpt.com</t>
+          <t>https://rakchamber.ae/</t>
         </is>
       </c>
     </row>
@@ -19816,7 +19816,7 @@
       </c>
       <c r="D87" s="16" t="inlineStr">
         <is>
-          <t>https://www.aopauae.com/events?utm_source=chatgpt.com</t>
+          <t>https://www.aopauae.com/events</t>
         </is>
       </c>
     </row>
@@ -19836,7 +19836,7 @@
       </c>
       <c r="D88" s="16" t="inlineStr">
         <is>
-          <t>https://www.abudhabichamber.ae/en?utm_source=chatgpt.com</t>
+          <t>https://www.abudhabichamber.ae/en</t>
         </is>
       </c>
     </row>
@@ -19856,7 +19856,7 @@
       </c>
       <c r="D89" s="16" t="inlineStr">
         <is>
-          <t>https://ajmanchamber.ae/en/archives/exhibitions-conferences/?utm_source=chatgpt.com</t>
+          <t>https://ajmanchamber.ae/en/archives/exhibitions-conferences/</t>
         </is>
       </c>
     </row>
@@ -20948,7 +20948,7 @@
       </c>
       <c r="D2" s="16" t="inlineStr">
         <is>
-          <t>https://www.taxinstitute.com.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.taxinstitute.com.au/events</t>
         </is>
       </c>
     </row>
@@ -20968,7 +20968,7 @@
       </c>
       <c r="D3" s="16" t="inlineStr">
         <is>
-          <t>https://www.cpaaustralia.com.au/professional-development/conferences-and-events?utm_source=chatgpt.com</t>
+          <t>https://www.cpaaustralia.com.au/professional-development/conferences-and-events</t>
         </is>
       </c>
     </row>
@@ -20988,7 +20988,7 @@
       </c>
       <c r="D4" s="16" t="inlineStr">
         <is>
-          <t>https://www.charteredaccountants.com.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.charteredaccountants.com.au/events</t>
         </is>
       </c>
     </row>
@@ -21008,7 +21008,7 @@
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>https://www.publicaccountants.org.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.publicaccountants.org.au/events</t>
         </is>
       </c>
     </row>
@@ -21028,7 +21028,7 @@
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>https://ifpa.com.au/events/?utm_source=chatgpt.com</t>
+          <t>https://ifpa.com.au/events/</t>
         </is>
       </c>
     </row>
@@ -21048,7 +21048,7 @@
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>https://ifa-australia.com.au/?utm_source=chatgpt.com</t>
+          <t>https://ifa-australia.com.au/</t>
         </is>
       </c>
     </row>
@@ -21068,7 +21068,7 @@
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>https://www.atma.com.au/?utm_source=chatgpt.com</t>
+          <t>https://www.atma.com.au/</t>
         </is>
       </c>
     </row>
@@ -21088,7 +21088,7 @@
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>https://faaa.au/events/?utm_source=chatgpt.com</t>
+          <t>https://faaa.au/events/</t>
         </is>
       </c>
     </row>
@@ -21108,7 +21108,7 @@
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>https://www.smsfassociation.com/events?utm_source=chatgpt.com</t>
+          <t>https://www.smsfassociation.com/events</t>
         </is>
       </c>
     </row>
@@ -21128,7 +21128,7 @@
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>https://www.aist.asn.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.aist.asn.au/events</t>
         </is>
       </c>
     </row>
@@ -21148,7 +21148,7 @@
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>https://www.afma.com.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.afma.com.au/events</t>
         </is>
       </c>
     </row>
@@ -21168,7 +21168,7 @@
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>https://www.ausbanking.org.au/events/?utm_source=chatgpt.com</t>
+          <t>https://www.ausbanking.org.au/events/</t>
         </is>
       </c>
     </row>
@@ -21188,7 +21188,7 @@
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>https://fsc.org.au/events?utm_source=chatgpt.com</t>
+          <t>https://fsc.org.au/events</t>
         </is>
       </c>
     </row>
@@ -21208,7 +21208,7 @@
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
-          <t>https://www.governanceinstitute.com.au/events/?utm_source=chatgpt.com</t>
+          <t>https://www.governanceinstitute.com.au/events/</t>
         </is>
       </c>
     </row>
@@ -21228,7 +21228,7 @@
       </c>
       <c r="D16" s="16" t="inlineStr">
         <is>
-          <t>https://arita.com.au/events?utm_source=chatgpt.com</t>
+          <t>https://arita.com.au/events</t>
         </is>
       </c>
     </row>
@@ -21248,7 +21248,7 @@
       </c>
       <c r="D17" s="16" t="inlineStr">
         <is>
-          <t>https://lawcouncil.au/events?utm_source=chatgpt.com</t>
+          <t>https://lawcouncil.au/events</t>
         </is>
       </c>
     </row>
@@ -21268,7 +21268,7 @@
       </c>
       <c r="D18" s="16" t="inlineStr">
         <is>
-          <t>https://www.lawsociety.com.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.lawsociety.com.au/events</t>
         </is>
       </c>
     </row>
@@ -21288,7 +21288,7 @@
       </c>
       <c r="D19" s="16" t="inlineStr">
         <is>
-          <t>https://www.liv.asn.au/Events?utm_source=chatgpt.com</t>
+          <t>https://www.liv.asn.au/Events</t>
         </is>
       </c>
     </row>
@@ -21308,7 +21308,7 @@
       </c>
       <c r="D20" s="16" t="inlineStr">
         <is>
-          <t>https://www.qls.com.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.qls.com.au/events</t>
         </is>
       </c>
     </row>
@@ -21328,7 +21328,7 @@
       </c>
       <c r="D21" s="16" t="inlineStr">
         <is>
-          <t>https://www.lawsocietysa.asn.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.lawsocietysa.asn.au/events</t>
         </is>
       </c>
     </row>
@@ -21348,7 +21348,7 @@
       </c>
       <c r="D22" s="16" t="inlineStr">
         <is>
-          <t>https://www.lawsocietywa.asn.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.lawsocietywa.asn.au/events</t>
         </is>
       </c>
     </row>
@@ -21368,7 +21368,7 @@
       </c>
       <c r="D23" s="16" t="inlineStr">
         <is>
-          <t>https://www.lst.org.au/events/?utm_source=chatgpt.com</t>
+          <t>https://www.lst.org.au/events/</t>
         </is>
       </c>
     </row>
@@ -21388,7 +21388,7 @@
       </c>
       <c r="D24" s="16" t="inlineStr">
         <is>
-          <t>https://lawsocietynt.com.au/events/?utm_source=chatgpt.com</t>
+          <t>https://lawsocietynt.com.au/events/</t>
         </is>
       </c>
     </row>
@@ -21408,7 +21408,7 @@
       </c>
       <c r="D25" s="16" t="inlineStr">
         <is>
-          <t>https://www.cla.org.au/Home?utm_source=chatgpt.com</t>
+          <t>https://www.cla.org.au/Home</t>
         </is>
       </c>
     </row>
@@ -21428,7 +21428,7 @@
       </c>
       <c r="D26" s="16" t="inlineStr">
         <is>
-          <t>https://www.academyoflaw.org.au/events-and-videos?utm_source=chatgpt.com</t>
+          <t>https://www.academyoflaw.org.au/events-and-videos</t>
         </is>
       </c>
     </row>
@@ -21448,7 +21448,7 @@
       </c>
       <c r="D27" s="16" t="inlineStr">
         <is>
-          <t>https://www.aala.org.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.aala.org.au/events</t>
         </is>
       </c>
     </row>
@@ -21468,7 +21468,7 @@
       </c>
       <c r="D28" s="16" t="inlineStr">
         <is>
-          <t>https://www.accaustralia.com.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.accaustralia.com.au/events</t>
         </is>
       </c>
     </row>
@@ -21488,7 +21488,7 @@
       </c>
       <c r="D29" s="16" t="inlineStr">
         <is>
-          <t>https://www.aicd.com.au/events.html?utm_source=chatgpt.com</t>
+          <t>https://www.aicd.com.au/events.html</t>
         </is>
       </c>
     </row>
@@ -21508,7 +21508,7 @@
       </c>
       <c r="D30" s="16" t="inlineStr">
         <is>
-          <t>https://www.aicm.com.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.aicm.com.au/events</t>
         </is>
       </c>
     </row>
@@ -21528,7 +21528,7 @@
       </c>
       <c r="D31" s="16" t="inlineStr">
         <is>
-          <t>https://www.financialcounsellingaustralia.org.au/events/?utm_source=chatgpt.com</t>
+          <t>https://www.financialcounsellingaustralia.org.au/events/</t>
         </is>
       </c>
     </row>
@@ -21548,7 +21548,7 @@
       </c>
       <c r="D32" s="16" t="inlineStr">
         <is>
-          <t>https://www.afp.org.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.afp.org.au/events</t>
         </is>
       </c>
     </row>
@@ -21568,7 +21568,7 @@
       </c>
       <c r="D33" s="16" t="inlineStr">
         <is>
-          <t>https://www.arpi.org.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.arpi.org.au/events</t>
         </is>
       </c>
     </row>
@@ -21588,7 +21588,7 @@
       </c>
       <c r="D34" s="16" t="inlineStr">
         <is>
-          <t>https://www.rmia.org.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.rmia.org.au/events</t>
         </is>
       </c>
     </row>
@@ -21608,7 +21608,7 @@
       </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
-          <t>https://www.aim.com.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.aim.com.au/events</t>
         </is>
       </c>
     </row>
@@ -21628,7 +21628,7 @@
       </c>
       <c r="D36" s="16" t="inlineStr">
         <is>
-          <t>https://aimwa.com/events/?utm_source=chatgpt.com</t>
+          <t>https://aimwa.com/events/</t>
         </is>
       </c>
     </row>
@@ -21648,7 +21648,7 @@
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>https://www.aiqs.com.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.aiqs.com.au/events</t>
         </is>
       </c>
     </row>
@@ -21668,7 +21668,7 @@
       </c>
       <c r="D38" s="16" t="inlineStr">
         <is>
-          <t>https://www.propertycouncil.com.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.propertycouncil.com.au/events</t>
         </is>
       </c>
     </row>
@@ -21688,7 +21688,7 @@
       </c>
       <c r="D39" s="16" t="inlineStr">
         <is>
-          <t>https://www.api.org.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.api.org.au/events</t>
         </is>
       </c>
     </row>
@@ -21708,7 +21708,7 @@
       </c>
       <c r="D40" s="16" t="inlineStr">
         <is>
-          <t>https://www.australianpayrollassociation.com.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.australianpayrollassociation.com.au/events</t>
         </is>
       </c>
     </row>
@@ -21728,7 +21728,7 @@
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>https://taps.associationonline.com.au/events/?utm_source=chatgpt.com</t>
+          <t>https://taps.associationonline.com.au/events/</t>
         </is>
       </c>
     </row>
@@ -21748,7 +21748,7 @@
       </c>
       <c r="D42" s="16" t="inlineStr">
         <is>
-          <t>https://aana.com.au/events/?utm_source=chatgpt.com</t>
+          <t>https://aana.com.au/events/</t>
         </is>
       </c>
     </row>
@@ -21768,7 +21768,7 @@
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>https://www.aicd.com.au/events.html?utm_source=chatgpt.com</t>
+          <t>https://www.aicd.com.au/events.html</t>
         </is>
       </c>
     </row>
@@ -21788,7 +21788,7 @@
       </c>
       <c r="D44" s="16" t="inlineStr">
         <is>
-          <t>https://www.abl.com.au/events/?utm_source=chatgpt.com</t>
+          <t>https://www.abl.com.au/events/</t>
         </is>
       </c>
     </row>
@@ -21808,7 +21808,7 @@
       </c>
       <c r="D45" s="16" t="inlineStr">
         <is>
-          <t>https://www.thomsonreuters.com.au/en-au/events.html?utm_source=chatgpt.com</t>
+          <t>https://www.thomsonreuters.com.au/en-au/events.html</t>
         </is>
       </c>
     </row>
@@ -21828,7 +21828,7 @@
       </c>
       <c r="D46" s="16" t="inlineStr">
         <is>
-          <t>https://www.tved.net.au/?utm_source=chatgpt.com</t>
+          <t>https://www.tved.net.au/</t>
         </is>
       </c>
     </row>
@@ -21848,7 +21848,7 @@
       </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>https://legalwiseseminars.com.au/events/?utm_source=chatgpt.com</t>
+          <t>https://legalwiseseminars.com.au/events/</t>
         </is>
       </c>
     </row>
@@ -21868,7 +21868,7 @@
       </c>
       <c r="D48" s="16" t="inlineStr">
         <is>
-          <t>https://www.leocussen.edu.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.leocussen.edu.au/events</t>
         </is>
       </c>
     </row>
@@ -21888,7 +21888,7 @@
       </c>
       <c r="D49" s="16" t="inlineStr">
         <is>
-          <t>https://www.collaw.edu.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.collaw.edu.au/events</t>
         </is>
       </c>
     </row>
@@ -21908,7 +21908,7 @@
       </c>
       <c r="D50" s="16" t="inlineStr">
         <is>
-          <t>https://www.aicd.com.au/events.html?utm_source=chatgpt.com</t>
+          <t>https://www.aicd.com.au/events.html</t>
         </is>
       </c>
     </row>
@@ -21928,7 +21928,7 @@
       </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
-          <t>https://www.aicd.com.au/events.html?utm_source=chatgpt.com</t>
+          <t>https://www.aicd.com.au/events.html</t>
         </is>
       </c>
     </row>
@@ -22748,7 +22748,7 @@
       </c>
       <c r="D92" s="16" t="inlineStr">
         <is>
-          <t>https://cfas.org.au/events/?utm_source=chatgpt.com</t>
+          <t>https://cfas.org.au/events/</t>
         </is>
       </c>
     </row>
@@ -22768,7 +22768,7 @@
       </c>
       <c r="D93" s="16" t="inlineStr">
         <is>
-          <t>https://erlaw.org.au/events/?utm_source=chatgpt.com</t>
+          <t>https://erlaw.org.au/events/</t>
         </is>
       </c>
     </row>
@@ -22788,7 +22788,7 @@
       </c>
       <c r="D94" s="16" t="inlineStr">
         <is>
-          <t>https://www.fintechaustralia.org.au/events/?utm_source=chatgpt.com</t>
+          <t>https://www.fintechaustralia.org.au/events/</t>
         </is>
       </c>
     </row>
@@ -22808,7 +22808,7 @@
       </c>
       <c r="D95" s="15" t="inlineStr">
         <is>
-          <t>https://www.mfaa.com.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.mfaa.com.au/events</t>
         </is>
       </c>
     </row>
@@ -22828,7 +22828,7 @@
       </c>
       <c r="D96" s="16" t="inlineStr">
         <is>
-          <t>https://shop.bfsla.org/?utm_source=chatgpt.com</t>
+          <t>https://shop.bfsla.org/</t>
         </is>
       </c>
     </row>
@@ -22848,7 +22848,7 @@
       </c>
       <c r="D97" s="16" t="inlineStr">
         <is>
-          <t>https://www.afia.asn.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.afia.asn.au/events</t>
         </is>
       </c>
     </row>
@@ -22868,7 +22868,7 @@
       </c>
       <c r="D98" s="16" t="inlineStr">
         <is>
-          <t>https://www.finpro.org.au/?utm_source=chatgpt.com</t>
+          <t>https://www.finpro.org.au/</t>
         </is>
       </c>
     </row>
@@ -22888,7 +22888,7 @@
       </c>
       <c r="D99" s="16" t="inlineStr">
         <is>
-          <t>https://pecbookings.eventsair.com/alla2026/?utm_source=chatgpt.com</t>
+          <t>https://pecbookings.eventsair.com/alla2026/</t>
         </is>
       </c>
     </row>
@@ -22908,7 +22908,7 @@
       </c>
       <c r="D100" s="16" t="inlineStr">
         <is>
-          <t>https://www.vscl.org.au/?utm_source=chatgpt.com</t>
+          <t>https://www.vscl.org.au/</t>
         </is>
       </c>
     </row>
@@ -22928,7 +22928,7 @@
       </c>
       <c r="D101" s="16" t="inlineStr">
         <is>
-          <t>https://www.claanz.org.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.claanz.org.au/events</t>
         </is>
       </c>
     </row>
@@ -22948,7 +22948,7 @@
       </c>
       <c r="D102" s="16" t="inlineStr">
         <is>
-          <t>https://www.probonocentre.org.au/news-media-2/events-and-conferences/?utm_source=chatgpt.com</t>
+          <t>https://www.probonocentre.org.au/news-media-2/events-and-conferences/</t>
         </is>
       </c>
     </row>
@@ -22968,7 +22968,7 @@
       </c>
       <c r="D103" s="16" t="inlineStr">
         <is>
-          <t>https://www.scla.org.au/events/?utm_source=chatgpt.com</t>
+          <t>https://www.scla.org.au/events/</t>
         </is>
       </c>
     </row>
@@ -22988,7 +22988,7 @@
       </c>
       <c r="D104" s="16" t="inlineStr">
         <is>
-          <t>https://www.tved.net.au/?utm_source=chatgpt.com</t>
+          <t>https://www.tved.net.au/</t>
         </is>
       </c>
     </row>
@@ -23008,7 +23008,7 @@
       </c>
       <c r="D105" s="16" t="inlineStr">
         <is>
-          <t>https://ifpa.com.au/events/?utm_source=chatgpt.com</t>
+          <t>https://ifpa.com.au/events/</t>
         </is>
       </c>
     </row>
@@ -23028,7 +23028,7 @@
       </c>
       <c r="D106" s="16" t="inlineStr">
         <is>
-          <t>https://www.afaanz.org/conference?utm_source=chatgpt.com</t>
+          <t>https://www.afaanz.org/conference</t>
         </is>
       </c>
     </row>
@@ -23048,7 +23048,7 @@
       </c>
       <c r="D107" s="16" t="inlineStr">
         <is>
-          <t>https://taps.associationonline.com.au/events/?utm_source=chatgpt.com</t>
+          <t>https://taps.associationonline.com.au/events/</t>
         </is>
       </c>
     </row>
@@ -23068,7 +23068,7 @@
       </c>
       <c r="D108" s="16" t="inlineStr">
         <is>
-          <t>https://www.api.org.au/events?utm_source=chatgpt.com</t>
+          <t>https://www.api.org.au/events</t>
         </is>
       </c>
     </row>

</xml_diff>